<commit_message>
Expand Charts into a full job cost board across every major PPR lane.
Subcontractor pie stays, but Charts now opens with doughnuts and bars for Direct craft, Indirect, per diem/travel, COE vs rentals, materials, overall forecast vs expended, hours, headcount, and the S-curve — the whole cost story, not one vendor tile.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
+++ b/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
@@ -17,7 +17,7 @@
     <sheet sheetId="8" name="_ChartData" state="veryHidden" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Charts'!$A1:$P45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Charts'!$A1:$X70</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Charts'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Cover'!$A1:$E18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Cover'!$1:$6</definedName>
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'T3 Export 15'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'T3 Export 16'!$A1:$I15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'T3 Export 16'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'_ChartData'!$A1:$L12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'_ChartData'!$A1:$AD13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'_ChartData'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="143">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -81,7 +81,7 @@
     <t>SAMPLE — synthetic hours and dollars for Look QA. Not a client actual.</t>
   </si>
   <si>
-    <t>Visuals first. Dense PPR field grid and Turnip ClientActual pastes follow as the working appendix.</t>
+    <t>Full job cost board — Direct, Indirect, Per diem/travel, Equipment, Rentals, Subs, Materials, hours. PPR field grid follows.</t>
   </si>
   <si>
     <t>Current Forecast $</t>
@@ -96,394 +96,400 @@
     <t>Hours To Go</t>
   </si>
   <si>
-    <t>Steel = live-pack estimate / budget  ·  Amber = Turnip expended  ·  Subcontractor doughnut from the live pack vendor sheet.</t>
+    <t>Steel = live-pack forecast  ·  Amber = Turnip expended  ·  Every major PPR cost lane has a graph. Dense field grid is on Total Project PPR.</t>
+  </si>
+  <si>
+    <t>board</t>
+  </si>
+  <si>
+    <t>(1) Total Project PPR  ·  Job SAMPLE-2026-017  ·  2026</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Detail</t>
+  </si>
+  <si>
+    <t>PPR snapshot</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Client</t>
+  </si>
+  <si>
+    <t>Sample Refinery</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>SAMPLE Boiler Outage PPR</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Wood River — Roxana, IL</t>
+  </si>
+  <si>
+    <t>Workhours Budget</t>
+  </si>
+  <si>
+    <t>Job #</t>
+  </si>
+  <si>
+    <t>SAMPLE-2026-017</t>
+  </si>
+  <si>
+    <t>Hours Expended To Date</t>
+  </si>
+  <si>
+    <t>Status Date</t>
+  </si>
+  <si>
+    <t>2026-09-03</t>
+  </si>
+  <si>
+    <t>Hours Earned To Date</t>
+  </si>
+  <si>
+    <t>Estimate status</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Prepared by</t>
+  </si>
+  <si>
+    <t>Hit Squad Project Controls</t>
+  </si>
+  <si>
+    <t>Performance To Date</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>SAMPLE status — invented hours and dollars only</t>
+  </si>
+  <si>
+    <t>Charts lead the package. Budget from this job’s live estimate pack. Actuals from Turnip T3 Export 15 / 16 through the Status Date. Yellow = Expended. Cyan = Earned.</t>
+  </si>
+  <si>
+    <t>Status Date 2026-09-03  ·  Status: In progress  ·  Prepared by: Hit Squad Project Controls  ·  Produced by Hit Squad Project Controls</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Dollars Budget</t>
+  </si>
+  <si>
+    <t>Wage Rate</t>
+  </si>
+  <si>
+    <t>Work Hours Expended</t>
+  </si>
+  <si>
+    <t>Dollars Expended</t>
+  </si>
+  <si>
+    <t>Work Hours Earned</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Hrs</t>
+  </si>
+  <si>
+    <t>$ / Hr</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Original</t>
+  </si>
+  <si>
+    <t>Revised</t>
+  </si>
+  <si>
+    <t>Current Forecast</t>
+  </si>
+  <si>
+    <t>Budget Rate</t>
+  </si>
+  <si>
+    <t>Actual Rate</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>To Date</t>
+  </si>
+  <si>
+    <t>To Go Forecast</t>
+  </si>
+  <si>
+    <t>DIRECT LABOR</t>
+  </si>
+  <si>
+    <t>Pipefitter Journeyman</t>
+  </si>
+  <si>
+    <t>Boilermaker Journeyman</t>
+  </si>
+  <si>
+    <t>Subtotal Direct Labor</t>
+  </si>
+  <si>
+    <t>INDIRECT LABOR</t>
+  </si>
+  <si>
+    <t>Foremen</t>
+  </si>
+  <si>
+    <t>Support</t>
+  </si>
+  <si>
+    <t>Staff</t>
+  </si>
+  <si>
+    <t>Per Diem</t>
+  </si>
+  <si>
+    <t>Mileage / Travel</t>
+  </si>
+  <si>
+    <t>Weather Delays</t>
+  </si>
+  <si>
+    <t>Onboarding</t>
+  </si>
+  <si>
+    <t>Subtotal Labor / PD</t>
+  </si>
+  <si>
+    <t>MATERIALS &amp; SUBCONTRACTS</t>
+  </si>
+  <si>
+    <t>Materials</t>
+  </si>
+  <si>
+    <t>Company Owned Equipment</t>
+  </si>
+  <si>
+    <t>Subcontractors</t>
+  </si>
+  <si>
+    <t>3rd Party General Rentals</t>
+  </si>
+  <si>
+    <t>Subtotal Material &amp; Subcontracts</t>
+  </si>
+  <si>
+    <t>TOTAL PROJECT</t>
+  </si>
+  <si>
+    <t>SAMPLE status — invented hours and dollars only  ·  Day-1 earned hours: Direct earned tracks expended (no P6 this pass). Support earned = Direct physical % complete × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
+  </si>
+  <si>
+    <t>Hours S-curve  ·  steel = live-pack estimate  ·  amber = T3 Export 16 spent</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Est hours</t>
+  </si>
+  <si>
+    <t>Act hours</t>
+  </si>
+  <si>
+    <t>Cum est hours</t>
+  </si>
+  <si>
+    <t>Cum act hours</t>
+  </si>
+  <si>
+    <t>Est headcount</t>
+  </si>
+  <si>
+    <t>Act headcount</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>2026-09-02</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>Cumulative hours — estimate vs actuals</t>
+  </si>
+  <si>
+    <t>Steel = live-pack estimate  ·  Amber = T3 Export 16 Units  ·  chart-ready columns D / E</t>
+  </si>
+  <si>
+    <t>Dated daily report log</t>
+  </si>
+  <si>
+    <t>Status date</t>
+  </si>
+  <si>
+    <t>Saved</t>
+  </si>
+  <si>
+    <t>Forecast $</t>
+  </si>
+  <si>
+    <t>Expended $</t>
+  </si>
+  <si>
+    <t>Budget hours</t>
+  </si>
+  <si>
+    <t>Expended hours</t>
+  </si>
+  <si>
+    <t>1970-01-01 00:00:00</t>
+  </si>
+  <si>
+    <t>SAMPLE day 1 — synthetic Turnip paste</t>
+  </si>
+  <si>
+    <t>T3 Export 15 — Client Cost Analysis  ·  Status Date 2026-09-03</t>
+  </si>
+  <si>
+    <t>ChargeCode</t>
+  </si>
+  <si>
+    <t>WO_Description</t>
+  </si>
+  <si>
+    <t>LaborTotal_ClientActual_Units</t>
+  </si>
+  <si>
+    <t>LaborTotal_ClientActual_Dollars</t>
+  </si>
+  <si>
+    <t>PD_ClientActual_Dollars</t>
+  </si>
+  <si>
+    <t>Other_ClientActual_Units</t>
+  </si>
+  <si>
+    <t>TotalDollars_ClientActual</t>
+  </si>
+  <si>
+    <t>Direct Labor</t>
+  </si>
+  <si>
+    <t>T3 Export 16 — Client Craft Analysis  ·  Status Date 2026-09-03</t>
+  </si>
+  <si>
+    <t>event_dt</t>
+  </si>
+  <si>
+    <t>craft</t>
+  </si>
+  <si>
+    <t>employee</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>ST_Units</t>
+  </si>
+  <si>
+    <t>OT_Units</t>
+  </si>
+  <si>
+    <t>DT_Units</t>
+  </si>
+  <si>
+    <t>Headcount</t>
+  </si>
+  <si>
+    <t>SAMPLE-101</t>
+  </si>
+  <si>
+    <t>SAMPLE-201</t>
+  </si>
+  <si>
+    <t>Firewatch</t>
+  </si>
+  <si>
+    <t>SAMPLE-301</t>
+  </si>
+  <si>
+    <t>Chart source — hidden helper</t>
+  </si>
+  <si>
+    <t>Ranges referenced by the Charts dashboard and Hrs S-curve.</t>
+  </si>
+  <si>
+    <t>Vendor</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Cost element</t>
+  </si>
+  <si>
+    <t>Direct craft</t>
+  </si>
+  <si>
+    <t>Indirect</t>
+  </si>
+  <si>
+    <t>Per diem / travel</t>
+  </si>
+  <si>
+    <t>Equipment / rentals</t>
+  </si>
+  <si>
+    <t>Materials / other</t>
+  </si>
+  <si>
+    <t>Craft</t>
+  </si>
+  <si>
+    <t>Hours</t>
   </si>
   <si>
     <t>SAMPLE NDE</t>
   </si>
   <si>
-    <t>(1) Total Project PPR  ·  Job SAMPLE-2026-017  ·  2026</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Detail</t>
-  </si>
-  <si>
-    <t>PPR snapshot</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Client</t>
-  </si>
-  <si>
-    <t>Sample Refinery</t>
-  </si>
-  <si>
-    <t>Job</t>
-  </si>
-  <si>
-    <t>SAMPLE Boiler Outage PPR</t>
-  </si>
-  <si>
-    <t>Site</t>
-  </si>
-  <si>
-    <t>Wood River — Roxana, IL</t>
-  </si>
-  <si>
-    <t>Workhours Budget</t>
-  </si>
-  <si>
-    <t>Job #</t>
-  </si>
-  <si>
-    <t>SAMPLE-2026-017</t>
-  </si>
-  <si>
-    <t>Hours Expended To Date</t>
-  </si>
-  <si>
-    <t>Status Date</t>
-  </si>
-  <si>
-    <t>2026-09-03</t>
-  </si>
-  <si>
-    <t>Hours Earned To Date</t>
-  </si>
-  <si>
-    <t>Estimate status</t>
-  </si>
-  <si>
-    <t>In progress</t>
-  </si>
-  <si>
-    <t>Prepared by</t>
-  </si>
-  <si>
-    <t>Hit Squad Project Controls</t>
-  </si>
-  <si>
-    <t>Performance To Date</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>SAMPLE status — invented hours and dollars only</t>
-  </si>
-  <si>
-    <t>Charts lead the package. Budget from this job’s live estimate pack. Actuals from Turnip T3 Export 15 / 16 through the Status Date. Yellow = Expended. Cyan = Earned.</t>
-  </si>
-  <si>
-    <t>Status Date 2026-09-03  ·  Status: In progress  ·  Prepared by: Hit Squad Project Controls  ·  Produced by Hit Squad Project Controls</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Dollars Budget</t>
-  </si>
-  <si>
-    <t>Wage Rate</t>
-  </si>
-  <si>
-    <t>Work Hours Expended</t>
-  </si>
-  <si>
-    <t>Dollars Expended</t>
-  </si>
-  <si>
-    <t>Work Hours Earned</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>$</t>
-  </si>
-  <si>
-    <t>Hrs</t>
-  </si>
-  <si>
-    <t>$ / Hr</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>Original</t>
-  </si>
-  <si>
-    <t>Revised</t>
-  </si>
-  <si>
-    <t>Current Forecast</t>
-  </si>
-  <si>
-    <t>Budget Rate</t>
-  </si>
-  <si>
-    <t>Actual Rate</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>To Date</t>
-  </si>
-  <si>
-    <t>To Go Forecast</t>
-  </si>
-  <si>
-    <t>DIRECT LABOR</t>
-  </si>
-  <si>
-    <t>Pipefitter Journeyman</t>
-  </si>
-  <si>
-    <t>Boilermaker Journeyman</t>
-  </si>
-  <si>
-    <t>Subtotal Direct Labor</t>
-  </si>
-  <si>
-    <t>INDIRECT LABOR</t>
-  </si>
-  <si>
-    <t>Foremen</t>
-  </si>
-  <si>
-    <t>Support</t>
-  </si>
-  <si>
-    <t>Staff</t>
-  </si>
-  <si>
-    <t>Per Diem</t>
-  </si>
-  <si>
-    <t>Mileage / Travel</t>
-  </si>
-  <si>
-    <t>Weather Delays</t>
-  </si>
-  <si>
-    <t>Onboarding</t>
-  </si>
-  <si>
-    <t>Subtotal Labor / PD</t>
-  </si>
-  <si>
-    <t>MATERIALS &amp; SUBCONTRACTS</t>
-  </si>
-  <si>
-    <t>Materials</t>
-  </si>
-  <si>
-    <t>Company Owned Equipment</t>
-  </si>
-  <si>
-    <t>Subcontractors</t>
-  </si>
-  <si>
-    <t>3rd Party General Rentals</t>
-  </si>
-  <si>
-    <t>Subtotal Material &amp; Subcontracts</t>
-  </si>
-  <si>
-    <t>TOTAL PROJECT</t>
-  </si>
-  <si>
-    <t>SAMPLE status — invented hours and dollars only  ·  Day-1 earned hours: Direct earned tracks expended (no P6 this pass). Support earned = Direct physical % complete × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
-  </si>
-  <si>
-    <t>Hours S-curve  ·  steel = live-pack estimate  ·  amber = T3 Export 16 spent</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Est hours</t>
-  </si>
-  <si>
-    <t>Act hours</t>
-  </si>
-  <si>
-    <t>Cum est hours</t>
-  </si>
-  <si>
-    <t>Cum act hours</t>
-  </si>
-  <si>
-    <t>Est headcount</t>
-  </si>
-  <si>
-    <t>Act headcount</t>
-  </si>
-  <si>
-    <t>2026-09-01</t>
-  </si>
-  <si>
-    <t>2026-09-02</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>Cumulative hours — estimate vs actuals</t>
-  </si>
-  <si>
-    <t>Steel = live-pack estimate  ·  Amber = T3 Export 16 Units  ·  chart-ready columns D / E</t>
-  </si>
-  <si>
-    <t>Dated daily report log</t>
-  </si>
-  <si>
-    <t>Status date</t>
-  </si>
-  <si>
-    <t>Saved</t>
-  </si>
-  <si>
-    <t>Forecast $</t>
-  </si>
-  <si>
-    <t>Expended $</t>
-  </si>
-  <si>
-    <t>Budget hours</t>
-  </si>
-  <si>
-    <t>Expended hours</t>
-  </si>
-  <si>
-    <t>1970-01-01 00:00:00</t>
-  </si>
-  <si>
-    <t>SAMPLE day 1 — synthetic Turnip paste</t>
-  </si>
-  <si>
-    <t>T3 Export 15 — Client Cost Analysis  ·  Status Date 2026-09-03</t>
-  </si>
-  <si>
-    <t>ChargeCode</t>
-  </si>
-  <si>
-    <t>WO_Description</t>
-  </si>
-  <si>
-    <t>LaborTotal_ClientActual_Units</t>
-  </si>
-  <si>
-    <t>LaborTotal_ClientActual_Dollars</t>
-  </si>
-  <si>
-    <t>PD_ClientActual_Dollars</t>
-  </si>
-  <si>
-    <t>Other_ClientActual_Units</t>
-  </si>
-  <si>
-    <t>TotalDollars_ClientActual</t>
-  </si>
-  <si>
-    <t>Direct Labor</t>
-  </si>
-  <si>
-    <t>T3 Export 16 — Client Craft Analysis  ·  Status Date 2026-09-03</t>
-  </si>
-  <si>
-    <t>event_dt</t>
-  </si>
-  <si>
-    <t>craft</t>
-  </si>
-  <si>
-    <t>employee</t>
-  </si>
-  <si>
-    <t>Units</t>
-  </si>
-  <si>
-    <t>ST_Units</t>
-  </si>
-  <si>
-    <t>OT_Units</t>
-  </si>
-  <si>
-    <t>DT_Units</t>
-  </si>
-  <si>
-    <t>Headcount</t>
-  </si>
-  <si>
-    <t>SAMPLE-101</t>
-  </si>
-  <si>
-    <t>SAMPLE-201</t>
-  </si>
-  <si>
-    <t>Firewatch</t>
-  </si>
-  <si>
-    <t>SAMPLE-301</t>
-  </si>
-  <si>
-    <t>Chart source — hidden helper</t>
-  </si>
-  <si>
-    <t>Ranges referenced by the Charts dashboard and Hrs S-curve.</t>
-  </si>
-  <si>
-    <t>Vendor</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>Cost element</t>
-  </si>
-  <si>
-    <t>Budget $</t>
-  </si>
-  <si>
-    <t>Actual $</t>
-  </si>
-  <si>
-    <t>PPR row</t>
-  </si>
-  <si>
-    <t>Craft</t>
-  </si>
-  <si>
-    <t>Hours</t>
-  </si>
-  <si>
     <t>SAMPLE Insulation</t>
   </si>
   <si>
-    <t>Indirect</t>
+    <t>Indirect labor</t>
+  </si>
+  <si>
+    <t>3rd Party Rentals</t>
   </si>
   <si>
     <t>SAMPLE Scaffold</t>
   </si>
   <si>
-    <t>Equipment</t>
-  </si>
-  <si>
     <t>SAMPLE Crane</t>
   </si>
   <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>3rd Party Rentals</t>
+    <t>Equipment (COE)</t>
   </si>
 </sst>
 </file>
@@ -972,7 +978,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Subcontractor costs — live pack by vendor</a:t>
+              <a:t>Job cost mix — Current Forecast by area</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -988,7 +994,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Subcontractor $</c:v>
+            <c:v>Job cost mix — Current Forecast by area</c:v>
           </c:tx>
           <c:dPt>
             <c:idx val="0"/>
@@ -1046,14 +1052,56 @@
               </a:ln>
             </c:spPr>
           </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B0F0"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C4922A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B6F73"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
           <c:cat>
             <c:strRef>
-              <c:f>'_ChartData'!$A$7:$A$10</c:f>
+              <c:f>'_ChartData'!$D$7:$D$13</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'_ChartData'!$B$7:$B$10</c:f>
+              <c:f>'_ChartData'!$E$7:$E$13</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1101,314 +1149,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1200" b="1"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="0F5F6D"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>Cost element mix — Current Forecast vs Expended</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'_ChartData'!$E$6:$E$6</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="0F5F6D"/>
-            </a:solidFill>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>'_ChartData'!$D$7:$D$12</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'_ChartData'!$E$7:$E$12</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'_ChartData'!$F$6:$F$6</c:f>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="E38B2A"/>
-            </a:solidFill>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>'_ChartData'!$D$7:$D$12</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'_ChartData'!$F$7:$F$12</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:dLbls>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="80"/>
-        <c:axId val="1"/>
-        <c:axId val="2"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="2"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="6350">
-              <a:solidFill>
-                <a:srgbClr val="8AA3A1"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1"/>
-        <c:crosses val="autoZero"/>
-      </c:valAx>
-      <c:spPr>
-        <a:solidFill>
-          <a:srgbClr val="F7FAF9"/>
-        </a:solidFill>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="0F5F6D"/>
-          </a:solidFill>
-        </a:ln>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln w="12700">
-      <a:solidFill>
-        <a:srgbClr val="0F5F6D"/>
-      </a:solidFill>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <c:roundedCorners val="0"/>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1200" b="1"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="0F5F6D"/>
-                </a:solidFill>
-                <a:latin typeface="Calibri"/>
-              </a:rPr>
-              <a:t>Dollars expended to date — major PPR rows</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Expended $</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="0F5F6D"/>
-            </a:solidFill>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>'_ChartData'!$H$7:$H$12</c:f>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'_ChartData'!$I$7:$I$12</c:f>
-            </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:dLbls>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="80"/>
-        <c:axId val="1"/>
-        <c:axId val="2"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="1"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="2"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="2"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="6350">
-              <a:solidFill>
-                <a:srgbClr val="8AA3A1"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
-        <c:majorTickMark val="out"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1"/>
-        <c:crosses val="autoZero"/>
-      </c:valAx>
-      <c:spPr>
-        <a:solidFill>
-          <a:srgbClr val="F7FAF9"/>
-        </a:solidFill>
-        <a:ln w="6350">
-          <a:solidFill>
-            <a:srgbClr val="0F5F6D"/>
-          </a:solidFill>
-        </a:ln>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="FFFFFF"/>
-    </a:solidFill>
-    <a:ln w="12700">
-      <a:solidFill>
-        <a:srgbClr val="0F5F6D"/>
-      </a:solidFill>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:roundedCorners val="0"/>
   <c:chart>
@@ -1458,12 +1199,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'_ChartData'!$K$7:$K$9</c:f>
+              <c:f>'_ChartData'!$AB$7:$AB$9</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'_ChartData'!$L$7:$L$9</c:f>
+              <c:f>'_ChartData'!$AC$7:$AC$9</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1547,7 +1288,146 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Peak headcount by craft — T3 Export 16</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Headcount</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F5F6D"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$AB$7:$AB$9</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$AD$7:$AD$9</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="8AA3A1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:roundedCorners val="0"/>
   <c:chart>
@@ -1736,6 +1616,1430 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Hours S-curve — live-pack estimate vs T3 Export 16 actuals</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Estimate hours</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Hrs S-curve'!$A$7:$A$10</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Hrs S-curve'!$D$7:$D$10</c:f>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Actual hours</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400">
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E38B2A"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Hrs S-curve'!$A$7:$A$10</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Hrs S-curve'!$E$7:$E$10</c:f>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="YYYY-MM-DD" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="8AA3A1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Forecast vs Expended — all cost areas</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$E$6:$E$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F5F6D"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$D$7:$D$13</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$E$7:$E$13</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$F$6:$F$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E38B2A"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$D$7:$D$13</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$F$7:$F$13</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="8AA3A1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Direct craft labor — by craft (Forecast $)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Direct craft labor — by craft (Forecast $)</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$H$7:$H$8</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$I$7:$I$8</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="58"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Indirect labor — Foremen / Support / Staff</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Indirect labor — Foremen / Support / Staff</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1A7A88"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$L$7:$L$9</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$M$7:$M$9</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="58"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Per diem and travel — Forecast vs Expended</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$Q$6:$Q$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F5F6D"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$P$7:$P$8</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$Q$7:$Q$8</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$R$6:$R$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E38B2A"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$P$7:$P$8</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$R$7:$R$8</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="8AA3A1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Subcontractor costs — live pack by vendor</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Subcontractor costs — live pack by vendor</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1A7A88"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="083943"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$A$7:$A$10</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$B$7:$B$10</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="58"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Equipment and rentals — COE vs 3rd Party</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$U$6:$U$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F5F6D"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$T$7:$T$8</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$U$7:$U$8</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'_ChartData'!$V$6:$V$6</c:f>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="E38B2A"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$T$7:$T$8</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$V$7:$V$8</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="80"/>
+        <c:axId val="1"/>
+        <c:axId val="2"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="2"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="8AA3A1"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Materials and other reimbursables — Forecast $</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Materials and other reimbursables — Forecast $</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1A7A88"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$X$7:$X$9</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$Y$7:$Y$9</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="58"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="0F5F6D"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Where the money went — expended by area</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Where the money went — expended by area</c:v>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0F5F6D"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="E38B2A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1A7A88"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="083943"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B0F0"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C4922A"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="5B6F73"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'_ChartData'!$D$7:$D$13</c:f>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'_ChartData'!$F$7:$F$13</c:f>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:numFmt formatCode="$#,##0" sourceLinked="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="58"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="F7FAF9"/>
+        </a:solidFill>
+        <a:ln w="6350">
+          <a:solidFill>
+            <a:srgbClr val="0F5F6D"/>
+          </a:solidFill>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="12700">
+      <a:solidFill>
+        <a:srgbClr val="0F5F6D"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1748,12 +3052,12 @@
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Subcontractor costs — live pack by vendor"/>
+        <xdr:cNvPr id="2" name="Job cost mix — Current Forecast by area"/>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks noGrp="1"/>
         </xdr:cNvGraphicFramePr>
@@ -1780,12 +3084,12 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Cost element mix — Current Forecast vs Expended"/>
+        <xdr:cNvPr id="3" name="Forecast vs Expended — all cost areas"/>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks noGrp="1"/>
         </xdr:cNvGraphicFramePr>
@@ -1804,20 +3108,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Dollars expended to date — major PPR rows"/>
+        <xdr:cNvPr id="4" name="Direct craft labor — by craft (Forecast $)"/>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks noGrp="1"/>
         </xdr:cNvGraphicFramePr>
@@ -1836,20 +3140,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Hours by craft — T3 Export 16 Units"/>
+        <xdr:cNvPr id="5" name="Indirect labor — Foremen / Support / Staff"/>
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks noGrp="1"/>
         </xdr:cNvGraphicFramePr>
@@ -1861,6 +3165,262 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Per diem and travel — Forecast vs Expended"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Subcontractor costs — live pack by vendor"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Equipment and rentals — COE vs 3rd Party"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Materials and other reimbursables — Forecast $"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="10" name="Where the money went — expended by area"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="11" name="Hours by craft — T3 Export 16 Units"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="12" name="Peak headcount by craft — T3 Export 16"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="13" name="Hours S-curve — live-pack estimate vs T3 Export 16 actuals"/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2232,7 +3792,7 @@
     <tabColor rgb="FFE38B2A"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:X70"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -2240,7 +3800,7 @@
     <col min="4" max="16384" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2259,8 +3819,16 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
-    </row>
-    <row r="2" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2279,8 +3847,16 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -2299,8 +3875,16 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-    </row>
-    <row r="4" ht="6" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -2319,8 +3903,16 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
-    </row>
-    <row r="5" ht="6" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -2339,8 +3931,16 @@
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
@@ -2359,8 +3959,16 @@
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>6</v>
       </c>
@@ -2379,8 +3987,16 @@
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
       <c r="P7" s="5"/>
-    </row>
-    <row r="8" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5"/>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
@@ -2405,8 +4021,16 @@
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="7"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <f>'Total Project PPR'!D29</f>
         <v>65135.600000000006</v>
@@ -2424,183 +4048,291 @@
         <v>176</v>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
       <c r="G11" s="11"/>
     </row>
-    <row r="12" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
       <c r="G12" s="11"/>
     </row>
-    <row r="13" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
       <c r="G13" s="11"/>
     </row>
-    <row r="14" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="G14" s="11"/>
     </row>
-    <row r="15" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
       <c r="G15" s="11"/>
     </row>
-    <row r="16" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
       <c r="G16" s="11"/>
     </row>
-    <row r="17" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
       <c r="G17" s="11"/>
     </row>
-    <row r="18" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
       <c r="G18" s="11"/>
     </row>
-    <row r="19" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
       <c r="G19" s="11"/>
     </row>
-    <row r="20" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
       <c r="G20" s="11"/>
     </row>
-    <row r="21" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
       <c r="G21" s="11"/>
     </row>
-    <row r="22" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
       <c r="G22" s="11"/>
     </row>
-    <row r="23" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" s="11"/>
       <c r="G23" s="11"/>
     </row>
-    <row r="24" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
       <c r="G24" s="11"/>
     </row>
-    <row r="25" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
       <c r="G25" s="11"/>
     </row>
-    <row r="26" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
       <c r="G26" s="11"/>
     </row>
-    <row r="27" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" s="11"/>
       <c r="G27" s="11"/>
     </row>
-    <row r="28" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" s="11"/>
       <c r="G28" s="11"/>
     </row>
-    <row r="29" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
       <c r="G29" s="11"/>
     </row>
-    <row r="30" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
       <c r="G30" s="11"/>
     </row>
-    <row r="31" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
       <c r="G31" s="11"/>
     </row>
-    <row r="32" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="11"/>
       <c r="G32" s="11"/>
     </row>
-    <row r="33" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
       <c r="G33" s="11"/>
     </row>
-    <row r="34" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" s="11"/>
       <c r="G34" s="11"/>
     </row>
-    <row r="35" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" s="11"/>
       <c r="G35" s="11"/>
     </row>
-    <row r="36" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="G36" s="11"/>
     </row>
-    <row r="37" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" s="11"/>
       <c r="G37" s="11"/>
     </row>
-    <row r="38" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" s="11"/>
       <c r="G38" s="11"/>
     </row>
-    <row r="39" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" s="11"/>
       <c r="G39" s="11"/>
     </row>
-    <row r="40" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" s="11"/>
       <c r="G40" s="11"/>
     </row>
-    <row r="41" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" s="11"/>
       <c r="G41" s="11"/>
     </row>
-    <row r="42" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
       <c r="G42" s="11"/>
     </row>
-    <row r="43" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
       <c r="G43" s="11"/>
     </row>
-    <row r="44" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
       <c r="G44" s="11"/>
     </row>
-    <row r="45" ht="16" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" s="5" t="s">
+    <row r="45" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A45" s="11"/>
+      <c r="G45" s="11"/>
+    </row>
+    <row r="46" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A46" s="11"/>
+      <c r="G46" s="11"/>
+    </row>
+    <row r="47" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A47" s="11"/>
+      <c r="G47" s="11"/>
+    </row>
+    <row r="48" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A48" s="11"/>
+      <c r="G48" s="11"/>
+    </row>
+    <row r="49" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A49" s="11"/>
+      <c r="G49" s="11"/>
+    </row>
+    <row r="50" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A50" s="11"/>
+      <c r="G50" s="11"/>
+    </row>
+    <row r="51" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A51" s="11"/>
+      <c r="G51" s="11"/>
+    </row>
+    <row r="52" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A52" s="11"/>
+      <c r="G52" s="11"/>
+    </row>
+    <row r="53" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A53" s="11"/>
+      <c r="G53" s="11"/>
+    </row>
+    <row r="54" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A54" s="11"/>
+      <c r="G54" s="11"/>
+    </row>
+    <row r="55" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A55" s="11"/>
+      <c r="G55" s="11"/>
+    </row>
+    <row r="56" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A56" s="11"/>
+      <c r="G56" s="11"/>
+    </row>
+    <row r="57" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A57" s="11"/>
+      <c r="G57" s="11"/>
+    </row>
+    <row r="58" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A58" s="11"/>
+      <c r="G58" s="11"/>
+    </row>
+    <row r="59" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A59" s="11"/>
+      <c r="G59" s="11"/>
+    </row>
+    <row r="60" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A60" s="11"/>
+      <c r="G60" s="11"/>
+    </row>
+    <row r="61" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A61" s="11"/>
+      <c r="G61" s="11"/>
+    </row>
+    <row r="62" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A62" s="11"/>
+      <c r="G62" s="11"/>
+    </row>
+    <row r="63" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A63" s="11"/>
+      <c r="G63" s="11"/>
+    </row>
+    <row r="64" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A64" s="11"/>
+      <c r="G64" s="11"/>
+    </row>
+    <row r="65" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A65" s="11"/>
+      <c r="G65" s="11"/>
+    </row>
+    <row r="66" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A66" s="11"/>
+      <c r="G66" s="11"/>
+    </row>
+    <row r="67" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A67" s="11"/>
+      <c r="G67" s="11"/>
+    </row>
+    <row r="68" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A68" s="11"/>
+      <c r="G68" s="11"/>
+    </row>
+    <row r="69" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A69" s="11"/>
+      <c r="G69" s="11"/>
+    </row>
+    <row r="70" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A70" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
-      <c r="L45" s="5"/>
-      <c r="M45" s="5"/>
-      <c r="N45" s="5"/>
-      <c r="O45" s="5"/>
-      <c r="P45" s="12" t="s">
+      <c r="B70" s="5"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+      <c r="I70" s="5"/>
+      <c r="J70" s="5"/>
+      <c r="K70" s="5"/>
+      <c r="L70" s="5"/>
+      <c r="M70" s="5"/>
+      <c r="N70" s="5"/>
+      <c r="O70" s="5"/>
+      <c r="P70" s="5"/>
+      <c r="Q70" s="5"/>
+      <c r="R70" s="5"/>
+      <c r="S70" s="5"/>
+      <c r="T70" s="5"/>
+      <c r="U70" s="5"/>
+      <c r="V70" s="5"/>
+      <c r="W70" s="5"/>
+      <c r="X70" s="12" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
   <mergeCells count="8">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A3:P3"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="A5:P5"/>
-    <mergeCell ref="A6:P6"/>
-    <mergeCell ref="A7:P7"/>
-    <mergeCell ref="A45:O45"/>
+    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="A2:X2"/>
+    <mergeCell ref="A3:X3"/>
+    <mergeCell ref="A4:X4"/>
+    <mergeCell ref="A5:X5"/>
+    <mergeCell ref="A6:X6"/>
+    <mergeCell ref="A7:X7"/>
+    <mergeCell ref="A70:W70"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="2"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;B HIT SQUAD / PROJECT CONTROLS &amp;C Charts &amp;R Confidential</oddHeader>
     <oddFooter>&amp;L Produced by Hit Squad Project Controls &amp;C &amp;D &amp;R Page &amp;P of &amp;N</oddFooter>
@@ -5775,20 +7507,28 @@
     <tabColor rgb="FF0F5F6D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:AD13"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="4" max="6" width="18" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="10" customWidth="1"/>
-    <col min="13" max="16384" width="9" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="18" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="14" width="18" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="18" width="18" customWidth="1"/>
+    <col min="20" max="20" width="11" customWidth="1"/>
+    <col min="21" max="22" width="18" customWidth="1"/>
+    <col min="24" max="24" width="11" customWidth="1"/>
+    <col min="25" max="26" width="18" customWidth="1"/>
+    <col min="28" max="28" width="11" customWidth="1"/>
+    <col min="29" max="30" width="10" customWidth="1"/>
+    <col min="31" max="16384" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -5803,8 +7543,26 @@
       <c r="J1" s="17"/>
       <c r="K1" s="17"/>
       <c r="L1" s="17"/>
-    </row>
-    <row r="2" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="X1" s="17"/>
+      <c r="Y1" s="17"/>
+      <c r="Z1" s="17"/>
+      <c r="AA1" s="17"/>
+      <c r="AB1" s="17"/>
+      <c r="AC1" s="17"/>
+      <c r="AD1" s="17"/>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="62" t="s">
         <v>124</v>
       </c>
@@ -5819,8 +7577,26 @@
       <c r="J2" s="62"/>
       <c r="K2" s="62"/>
       <c r="L2" s="62"/>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+      <c r="U2" s="62"/>
+      <c r="V2" s="62"/>
+      <c r="W2" s="62"/>
+      <c r="X2" s="62"/>
+      <c r="Y2" s="62"/>
+      <c r="Z2" s="62"/>
+      <c r="AA2" s="62"/>
+      <c r="AB2" s="62"/>
+      <c r="AC2" s="62"/>
+      <c r="AD2" s="62"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
         <v>125</v>
       </c>
@@ -5835,8 +7611,26 @@
       <c r="J3" s="63"/>
       <c r="K3" s="63"/>
       <c r="L3" s="63"/>
-    </row>
-    <row r="4" ht="6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" s="63"/>
+      <c r="N3" s="63"/>
+      <c r="O3" s="63"/>
+      <c r="P3" s="63"/>
+      <c r="Q3" s="63"/>
+      <c r="R3" s="63"/>
+      <c r="S3" s="63"/>
+      <c r="T3" s="63"/>
+      <c r="U3" s="63"/>
+      <c r="V3" s="63"/>
+      <c r="W3" s="63"/>
+      <c r="X3" s="63"/>
+      <c r="Y3" s="63"/>
+      <c r="Z3" s="63"/>
+      <c r="AA3" s="63"/>
+      <c r="AB3" s="63"/>
+      <c r="AC3" s="63"/>
+      <c r="AD3" s="63"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="64"/>
       <c r="B4" s="64"/>
       <c r="C4" s="64"/>
@@ -5849,8 +7643,26 @@
       <c r="J4" s="64"/>
       <c r="K4" s="64"/>
       <c r="L4" s="64"/>
-    </row>
-    <row r="5" ht="6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" s="64"/>
+      <c r="N4" s="64"/>
+      <c r="O4" s="64"/>
+      <c r="P4" s="64"/>
+      <c r="Q4" s="64"/>
+      <c r="R4" s="64"/>
+      <c r="S4" s="64"/>
+      <c r="T4" s="64"/>
+      <c r="U4" s="64"/>
+      <c r="V4" s="64"/>
+      <c r="W4" s="64"/>
+      <c r="X4" s="64"/>
+      <c r="Y4" s="64"/>
+      <c r="Z4" s="64"/>
+      <c r="AA4" s="64"/>
+      <c r="AB4" s="64"/>
+      <c r="AC4" s="64"/>
+      <c r="AD4" s="64"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="64"/>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -5863,8 +7675,26 @@
       <c r="J5" s="64"/>
       <c r="K5" s="64"/>
       <c r="L5" s="64"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" s="64"/>
+      <c r="N5" s="64"/>
+      <c r="O5" s="64"/>
+      <c r="P5" s="64"/>
+      <c r="Q5" s="64"/>
+      <c r="R5" s="64"/>
+      <c r="S5" s="64"/>
+      <c r="T5" s="64"/>
+      <c r="U5" s="64"/>
+      <c r="V5" s="64"/>
+      <c r="W5" s="64"/>
+      <c r="X5" s="64"/>
+      <c r="Y5" s="64"/>
+      <c r="Z5" s="64"/>
+      <c r="AA5" s="64"/>
+      <c r="AB5" s="64"/>
+      <c r="AC5" s="64"/>
+      <c r="AD5" s="64"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="65" t="s">
         <v>126</v>
       </c>
@@ -5876,29 +7706,75 @@
         <v>128</v>
       </c>
       <c r="E6" s="65" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
       <c r="F6" s="65" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="G6" s="83"/>
       <c r="H6" s="65" t="s">
+        <v>129</v>
+      </c>
+      <c r="I6" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="J6" s="65" t="s">
+        <v>97</v>
+      </c>
+      <c r="K6" s="83"/>
+      <c r="L6" s="65" t="s">
+        <v>130</v>
+      </c>
+      <c r="M6" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="N6" s="65" t="s">
+        <v>97</v>
+      </c>
+      <c r="O6" s="83"/>
+      <c r="P6" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="65" t="s">
+      <c r="Q6" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="R6" s="65" t="s">
         <v>97</v>
       </c>
-      <c r="J6" s="83"/>
-      <c r="K6" s="65" t="s">
+      <c r="S6" s="83"/>
+      <c r="T6" s="65" t="s">
         <v>132</v>
       </c>
-      <c r="L6" s="65" t="s">
+      <c r="U6" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="V6" s="65" t="s">
+        <v>97</v>
+      </c>
+      <c r="W6" s="83"/>
+      <c r="X6" s="65" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="Y6" s="65" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z6" s="65" t="s">
+        <v>97</v>
+      </c>
+      <c r="AA6" s="83"/>
+      <c r="AB6" s="65" t="s">
+        <v>134</v>
+      </c>
+      <c r="AC6" s="65" t="s">
+        <v>135</v>
+      </c>
+      <c r="AD6" s="65" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="66" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="B7" s="76">
         <v>6500</v>
@@ -5917,181 +7793,401 @@
       </c>
       <c r="G7" s="84"/>
       <c r="H7" s="75" t="s">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="I7" s="76">
-        <f>'Total Project PPR'!M13</f>
-        <v>18480</v>
-      </c>
-      <c r="J7" s="84"/>
-      <c r="K7" s="75" t="s">
+        <f>'Total Project PPR'!D11</f>
+        <v>17152.32</v>
+      </c>
+      <c r="J7" s="76">
+        <f>'Total Project PPR'!M11</f>
+        <v>10560</v>
+      </c>
+      <c r="K7" s="84"/>
+      <c r="L7" s="75" t="s">
+        <v>64</v>
+      </c>
+      <c r="M7" s="76">
+        <f>'Total Project PPR'!D15</f>
+        <v>4548.96</v>
+      </c>
+      <c r="N7" s="76">
+        <f>'Total Project PPR'!M15</f>
+        <v>3120</v>
+      </c>
+      <c r="O7" s="84"/>
+      <c r="P7" s="75" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q7" s="76">
+        <f>'Total Project PPR'!D18</f>
+        <v>2640</v>
+      </c>
+      <c r="R7" s="76">
+        <f>'Total Project PPR'!M18</f>
+        <v>1820</v>
+      </c>
+      <c r="S7" s="84"/>
+      <c r="T7" s="75" t="s">
+        <v>74</v>
+      </c>
+      <c r="U7" s="76">
+        <f>'Total Project PPR'!D25</f>
+        <v>0</v>
+      </c>
+      <c r="V7" s="76">
+        <f>'Total Project PPR'!M25</f>
+        <v>0</v>
+      </c>
+      <c r="W7" s="84"/>
+      <c r="X7" s="75" t="s">
+        <v>73</v>
+      </c>
+      <c r="Y7" s="76">
+        <f>'Total Project PPR'!D24</f>
+        <v>1020</v>
+      </c>
+      <c r="Z7" s="76">
+        <f>'Total Project PPR'!M24</f>
+        <v>0</v>
+      </c>
+      <c r="AA7" s="84"/>
+      <c r="AB7" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="L7" s="67">
+      <c r="AC7" s="67">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="AD7" s="67">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="68" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B8" s="78">
         <v>4200</v>
       </c>
       <c r="C8" s="86"/>
       <c r="D8" s="72" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E8" s="78">
-        <f>SUM('Total Project PPR'!D15,'Total Project PPR'!D16,'Total Project PPR'!D17,'Total Project PPR'!D18,'Total Project PPR'!D19,'Total Project PPR'!D20,'Total Project PPR'!D21)</f>
-        <v>12292.08</v>
+        <f>SUM('Total Project PPR'!D15,'Total Project PPR'!D16,'Total Project PPR'!D17)</f>
+        <v>9372.08</v>
       </c>
       <c r="F8" s="78">
-        <f>SUM('Total Project PPR'!M15,'Total Project PPR'!M16,'Total Project PPR'!M17,'Total Project PPR'!M18,'Total Project PPR'!M19,'Total Project PPR'!M20,'Total Project PPR'!M21)</f>
-        <v>12380</v>
+        <f>SUM('Total Project PPR'!M15,'Total Project PPR'!M16,'Total Project PPR'!M17)</f>
+        <v>10560</v>
       </c>
       <c r="G8" s="86"/>
       <c r="H8" s="77" t="s">
-        <v>135</v>
+        <v>61</v>
       </c>
       <c r="I8" s="78">
-        <f>SUM('Total Project PPR'!M15,'Total Project PPR'!M16,'Total Project PPR'!M17,'Total Project PPR'!M18,'Total Project PPR'!M19,'Total Project PPR'!M20,'Total Project PPR'!M21)</f>
-        <v>12380</v>
-      </c>
-      <c r="J8" s="86"/>
-      <c r="K8" s="77" t="s">
+        <f>'Total Project PPR'!D12</f>
+        <v>14071.2</v>
+      </c>
+      <c r="J8" s="78">
+        <f>'Total Project PPR'!M12</f>
+        <v>7920</v>
+      </c>
+      <c r="K8" s="86"/>
+      <c r="L8" s="77" t="s">
+        <v>65</v>
+      </c>
+      <c r="M8" s="78">
+        <f>'Total Project PPR'!D16</f>
+        <v>0</v>
+      </c>
+      <c r="N8" s="78">
+        <f>'Total Project PPR'!M16</f>
+        <v>3840</v>
+      </c>
+      <c r="O8" s="86"/>
+      <c r="P8" s="77" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q8" s="78">
+        <f>'Total Project PPR'!D19</f>
+        <v>280</v>
+      </c>
+      <c r="R8" s="78">
+        <f>'Total Project PPR'!M19</f>
+        <v>0</v>
+      </c>
+      <c r="S8" s="86"/>
+      <c r="T8" s="77" t="s">
+        <v>139</v>
+      </c>
+      <c r="U8" s="78">
+        <f>'Total Project PPR'!D27</f>
+        <v>2400</v>
+      </c>
+      <c r="V8" s="78">
+        <f>'Total Project PPR'!M27</f>
+        <v>0</v>
+      </c>
+      <c r="W8" s="86"/>
+      <c r="X8" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y8" s="78">
+        <f>'Total Project PPR'!D20</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="78">
+        <f>'Total Project PPR'!M20</f>
+        <v>0</v>
+      </c>
+      <c r="AA8" s="86"/>
+      <c r="AB8" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="L8" s="69">
+      <c r="AC8" s="69">
         <v>68</v>
       </c>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="AD8" s="69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="66" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B9" s="76">
         <v>3800</v>
       </c>
       <c r="C9" s="84"/>
       <c r="D9" s="85" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E9" s="76">
-        <f>'Total Project PPR'!D25</f>
-        <v>0</v>
+        <f>SUM('Total Project PPR'!D18,'Total Project PPR'!D19)</f>
+        <v>2920</v>
       </c>
       <c r="F9" s="76">
-        <f>'Total Project PPR'!M25</f>
-        <v>0</v>
+        <f>SUM('Total Project PPR'!M18,'Total Project PPR'!M19)</f>
+        <v>1820</v>
       </c>
       <c r="G9" s="84"/>
-      <c r="H9" s="75" t="s">
-        <v>137</v>
-      </c>
-      <c r="I9" s="76">
-        <f>'Total Project PPR'!M25</f>
-        <v>0</v>
-      </c>
-      <c r="J9" s="84"/>
-      <c r="K9" s="75" t="s">
+      <c r="H9" s="84"/>
+      <c r="I9" s="71"/>
+      <c r="J9" s="71"/>
+      <c r="K9" s="84"/>
+      <c r="L9" s="75" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="76">
+        <f>'Total Project PPR'!D17</f>
+        <v>4823.12</v>
+      </c>
+      <c r="N9" s="76">
+        <f>'Total Project PPR'!M17</f>
+        <v>3600</v>
+      </c>
+      <c r="O9" s="84"/>
+      <c r="P9" s="84"/>
+      <c r="Q9" s="71"/>
+      <c r="R9" s="71"/>
+      <c r="S9" s="84"/>
+      <c r="T9" s="84"/>
+      <c r="U9" s="71"/>
+      <c r="V9" s="71"/>
+      <c r="W9" s="84"/>
+      <c r="X9" s="75" t="s">
+        <v>70</v>
+      </c>
+      <c r="Y9" s="76">
+        <f>'Total Project PPR'!D21</f>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="76">
+        <f>'Total Project PPR'!M21</f>
+        <v>0</v>
+      </c>
+      <c r="AA9" s="84"/>
+      <c r="AB9" s="75" t="s">
         <v>122</v>
       </c>
-      <c r="L9" s="67">
+      <c r="AC9" s="67">
         <v>48</v>
       </c>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="AD9" s="67">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="68" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B10" s="78">
         <v>3700</v>
       </c>
       <c r="C10" s="86"/>
       <c r="D10" s="72" t="s">
-        <v>75</v>
+        <v>142</v>
       </c>
       <c r="E10" s="78">
-        <f>'Total Project PPR'!D26</f>
-        <v>18200</v>
+        <f>'Total Project PPR'!D25</f>
+        <v>0</v>
       </c>
       <c r="F10" s="78">
-        <f>'Total Project PPR'!M26</f>
-        <v>8200</v>
+        <f>'Total Project PPR'!M25</f>
+        <v>0</v>
       </c>
       <c r="G10" s="86"/>
-      <c r="H10" s="77" t="s">
-        <v>75</v>
-      </c>
-      <c r="I10" s="78">
-        <f>'Total Project PPR'!M26</f>
-        <v>8200</v>
-      </c>
-      <c r="J10" s="86"/>
+      <c r="H10" s="86"/>
+      <c r="I10" s="74"/>
+      <c r="J10" s="74"/>
       <c r="K10" s="86"/>
-      <c r="L10" s="74"/>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L10" s="86"/>
+      <c r="M10" s="74"/>
+      <c r="N10" s="74"/>
+      <c r="O10" s="86"/>
+      <c r="P10" s="86"/>
+      <c r="Q10" s="74"/>
+      <c r="R10" s="74"/>
+      <c r="S10" s="86"/>
+      <c r="T10" s="86"/>
+      <c r="U10" s="74"/>
+      <c r="V10" s="74"/>
+      <c r="W10" s="86"/>
+      <c r="X10" s="86"/>
+      <c r="Y10" s="74"/>
+      <c r="Z10" s="74"/>
+      <c r="AA10" s="86"/>
+      <c r="AB10" s="86"/>
+      <c r="AC10" s="74"/>
+      <c r="AD10" s="74"/>
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="71"/>
       <c r="C11" s="84"/>
       <c r="D11" s="85" t="s">
-        <v>73</v>
+        <v>139</v>
       </c>
       <c r="E11" s="76">
-        <f>'Total Project PPR'!D24</f>
-        <v>1020</v>
+        <f>'Total Project PPR'!D27</f>
+        <v>2400</v>
       </c>
       <c r="F11" s="76">
-        <f>'Total Project PPR'!M24</f>
+        <f>'Total Project PPR'!M27</f>
         <v>0</v>
       </c>
       <c r="G11" s="84"/>
-      <c r="H11" s="75" t="s">
-        <v>73</v>
-      </c>
-      <c r="I11" s="76">
-        <f>'Total Project PPR'!M24</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="84"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="71"/>
+      <c r="J11" s="71"/>
       <c r="K11" s="84"/>
-      <c r="L11" s="71"/>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L11" s="84"/>
+      <c r="M11" s="71"/>
+      <c r="N11" s="71"/>
+      <c r="O11" s="84"/>
+      <c r="P11" s="84"/>
+      <c r="Q11" s="71"/>
+      <c r="R11" s="71"/>
+      <c r="S11" s="84"/>
+      <c r="T11" s="84"/>
+      <c r="U11" s="71"/>
+      <c r="V11" s="71"/>
+      <c r="W11" s="84"/>
+      <c r="X11" s="84"/>
+      <c r="Y11" s="71"/>
+      <c r="Z11" s="71"/>
+      <c r="AA11" s="84"/>
+      <c r="AB11" s="84"/>
+      <c r="AC11" s="71"/>
+      <c r="AD11" s="71"/>
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="73"/>
       <c r="B12" s="74"/>
       <c r="C12" s="86"/>
       <c r="D12" s="72" t="s">
-        <v>139</v>
+        <v>75</v>
       </c>
       <c r="E12" s="78">
-        <f>'Total Project PPR'!D27</f>
-        <v>2400</v>
+        <f>'Total Project PPR'!D26</f>
+        <v>18200</v>
       </c>
       <c r="F12" s="78">
-        <f>'Total Project PPR'!M27</f>
-        <v>0</v>
+        <f>'Total Project PPR'!M26</f>
+        <v>8200</v>
       </c>
       <c r="G12" s="86"/>
-      <c r="H12" s="77" t="s">
-        <v>140</v>
-      </c>
-      <c r="I12" s="78">
-        <f>'Total Project PPR'!M27</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="86"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="74"/>
+      <c r="J12" s="74"/>
       <c r="K12" s="86"/>
-      <c r="L12" s="74"/>
+      <c r="L12" s="86"/>
+      <c r="M12" s="74"/>
+      <c r="N12" s="74"/>
+      <c r="O12" s="86"/>
+      <c r="P12" s="86"/>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
+      <c r="S12" s="86"/>
+      <c r="T12" s="86"/>
+      <c r="U12" s="74"/>
+      <c r="V12" s="74"/>
+      <c r="W12" s="86"/>
+      <c r="X12" s="86"/>
+      <c r="Y12" s="74"/>
+      <c r="Z12" s="74"/>
+      <c r="AA12" s="86"/>
+      <c r="AB12" s="86"/>
+      <c r="AC12" s="74"/>
+      <c r="AD12" s="74"/>
+    </row>
+    <row r="13" ht="16" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A13" s="70"/>
+      <c r="B13" s="71"/>
+      <c r="C13" s="84"/>
+      <c r="D13" s="85" t="s">
+        <v>133</v>
+      </c>
+      <c r="E13" s="76">
+        <f>SUM('Total Project PPR'!D24,'Total Project PPR'!D20,'Total Project PPR'!D21)</f>
+        <v>1020</v>
+      </c>
+      <c r="F13" s="76">
+        <f>SUM('Total Project PPR'!M24,'Total Project PPR'!M20,'Total Project PPR'!M21)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="84"/>
+      <c r="H13" s="84"/>
+      <c r="I13" s="71"/>
+      <c r="J13" s="71"/>
+      <c r="K13" s="84"/>
+      <c r="L13" s="84"/>
+      <c r="M13" s="71"/>
+      <c r="N13" s="71"/>
+      <c r="O13" s="84"/>
+      <c r="P13" s="84"/>
+      <c r="Q13" s="71"/>
+      <c r="R13" s="71"/>
+      <c r="S13" s="84"/>
+      <c r="T13" s="84"/>
+      <c r="U13" s="71"/>
+      <c r="V13" s="71"/>
+      <c r="W13" s="84"/>
+      <c r="X13" s="84"/>
+      <c r="Y13" s="71"/>
+      <c r="Z13" s="71"/>
+      <c r="AA13" s="84"/>
+      <c r="AB13" s="84"/>
+      <c r="AC13" s="71"/>
+      <c r="AD13" s="71"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
   <mergeCells count="3">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A1:AD1"/>
+    <mergeCell ref="A2:AD2"/>
+    <mergeCell ref="A3:AD3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>

</xml_diff>

<commit_message>
Add Schedule / Progress KPI entry so PPR earned uses scheduler hours.
Cost report can now store to-date earned workhours (plus optional daily, physical %, and unit rows) on the vault-backed book and daily snapshot. Excel Earned / % Complete bind to those KPIs when present and keep the Day-1 expended stand-in only when the fields are empty. SAMPLE uses distinct scheduler earned so cyan earned no longer copies yellow expended.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
+++ b/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
@@ -52,7 +52,7 @@
             <sz val="9"/>
             <rFont val="Calibri"/>
           </rPr>
-          <t>Day-1 earned hours: Direct earned tracks expended (no P6 this pass). Support earned = Direct physical % complete × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
+          <t>Earned hours from scheduler KPI on Cost report. Physical % = earned / Direct budget hours (hours win if % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
         </r>
       </text>
     </comment>
@@ -300,7 +300,7 @@
     <t>TOTAL PROJECT</t>
   </si>
   <si>
-    <t>SAMPLE status — invented hours and dollars only  ·  Day-1 earned hours: Direct earned tracks expended (no P6 this pass). Support earned = Direct physical % complete × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
+    <t>SAMPLE status — invented hours and dollars only  ·  Earned hours from scheduler KPI on Cost report. Physical % = earned / Direct budget hours (hours win if % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
   </si>
   <si>
     <t>Hours S-curve  ·  steel = live-pack estimate  ·  amber = T3 Export 16 spent</t>
@@ -4041,11 +4041,11 @@
       </c>
       <c r="E9" s="9">
         <f>'Total Project PPR'!Q29</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="G9" s="10">
         <f>'Total Project PPR'!T29</f>
-        <v>176</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="E13" s="13">
         <f>'Total Project PPR'!O29</f>
-        <v>264</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4516,7 +4516,7 @@
       </c>
       <c r="E14" s="9">
         <f>'Total Project PPR'!Q29</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="E15" s="14">
         <f>'Total Project PPR'!S29</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="E16" s="16">
         <f>'Total Project PPR'!T29</f>
-        <v>176</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25"/>
@@ -4952,18 +4952,18 @@
         <v>10560</v>
       </c>
       <c r="N11" s="32">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="O11" s="32">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="P11" s="33">
         <f>IF(G11=0,0,N11/G11)</f>
-        <v>0.375</v>
+        <v>0.15</v>
       </c>
       <c r="Q11" s="33">
         <f>IF(G11=0,0,O11/G11)</f>
-        <v>0.625</v>
+        <v>0.45</v>
       </c>
       <c r="R11" s="31">
         <f>D11-M11</f>
@@ -4971,11 +4971,11 @@
       </c>
       <c r="S11" s="34">
         <f>IF(K11=0,0,O11/K11)</f>
-        <v>1</v>
+        <v>0.72</v>
       </c>
       <c r="T11" s="35">
         <f>G11-O11</f>
-        <v>60</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5021,18 +5021,18 @@
         <v>7920</v>
       </c>
       <c r="N12" s="38">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="O12" s="38">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="P12" s="39">
         <f>IF(G12=0,0,N12/G12)</f>
-        <v>0.31666666666666665</v>
+        <v>0.15</v>
       </c>
       <c r="Q12" s="39">
         <f>IF(G12=0,0,O12/G12)</f>
-        <v>0.5666666666666667</v>
+        <v>0.45</v>
       </c>
       <c r="R12" s="37">
         <f>D12-M12</f>
@@ -5040,11 +5040,11 @@
       </c>
       <c r="S12" s="40">
         <f>IF(K12=0,0,O12/K12)</f>
-        <v>1</v>
+        <v>0.7941176470588235</v>
       </c>
       <c r="T12" s="41">
         <f>G12-O12</f>
-        <v>52</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5101,19 +5101,19 @@
       </c>
       <c r="N13" s="44">
         <f>SUM(N11,N12)</f>
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="O13" s="44">
         <f>SUM(O11,O12)</f>
-        <v>168</v>
+        <v>126</v>
       </c>
       <c r="P13" s="45">
         <f>IF(G13=0,0,N13/G13)</f>
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="Q13" s="45">
         <f>IF(G13=0,0,O13/G13)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R13" s="43">
         <f>D13-M13</f>
@@ -5121,11 +5121,11 @@
       </c>
       <c r="S13" s="46">
         <f>IF(K13=0,0,O13/K13)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T13" s="47">
         <f>G13-O13</f>
-        <v>112</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5195,18 +5195,18 @@
         <v>3120</v>
       </c>
       <c r="N15" s="32">
-        <v>12</v>
+        <v>9.6</v>
       </c>
       <c r="O15" s="32">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P15" s="33">
         <f>IF(G15=0,0,N15/G15)</f>
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="Q15" s="33">
         <f>IF(G15=0,0,O15/G15)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R15" s="31">
         <f>D15-M15</f>
@@ -5214,11 +5214,11 @@
       </c>
       <c r="S15" s="34">
         <f>IF(K15=0,0,O15/K15)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T15" s="35">
         <f>G15-O15</f>
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5264,18 +5264,18 @@
         <v>3840</v>
       </c>
       <c r="N16" s="38">
-        <v>24</v>
+        <v>19.2</v>
       </c>
       <c r="O16" s="38">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="P16" s="39">
         <f>IF(G16=0,0,N16/G16)</f>
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="Q16" s="39">
         <f>IF(G16=0,0,O16/G16)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R16" s="37">
         <f>D16-M16</f>
@@ -5283,11 +5283,11 @@
       </c>
       <c r="S16" s="40">
         <f>IF(K16=0,0,O16/K16)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T16" s="41">
         <f>G16-O16</f>
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5333,18 +5333,18 @@
         <v>3600</v>
       </c>
       <c r="N17" s="32">
-        <v>12</v>
+        <v>9.6</v>
       </c>
       <c r="O17" s="32">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="P17" s="33">
         <f>IF(G17=0,0,N17/G17)</f>
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="Q17" s="33">
         <f>IF(G17=0,0,O17/G17)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R17" s="31">
         <f>D17-M17</f>
@@ -5352,11 +5352,11 @@
       </c>
       <c r="S17" s="34">
         <f>IF(K17=0,0,O17/K17)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T17" s="35">
         <f>G17-O17</f>
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -5689,19 +5689,19 @@
       </c>
       <c r="N22" s="44">
         <f>SUM(N11,N12,N15,N16,N17,N18,N19,N20,N21)</f>
-        <v>146</v>
+        <v>80.39999999999999</v>
       </c>
       <c r="O22" s="44">
         <f>SUM(O11,O12,O15,O16,O17,O18,O19,O20,O21)</f>
-        <v>264</v>
+        <v>198</v>
       </c>
       <c r="P22" s="45">
         <f>IF(G22=0,0,N22/G22)</f>
-        <v>0.33181818181818185</v>
+        <v>0.1827272727272727</v>
       </c>
       <c r="Q22" s="45">
         <f>IF(G22=0,0,O22/G22)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R22" s="43">
         <f>D22-M22</f>
@@ -5709,11 +5709,11 @@
       </c>
       <c r="S22" s="46">
         <f>IF(K22=0,0,O22/K22)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T22" s="47">
         <f>G22-O22</f>
-        <v>176</v>
+        <v>242</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -6151,19 +6151,19 @@
       </c>
       <c r="N29" s="55">
         <f>SUM(N22,N28)</f>
-        <v>146</v>
+        <v>80.39999999999999</v>
       </c>
       <c r="O29" s="55">
         <f>SUM(O22,O28)</f>
-        <v>264</v>
+        <v>198</v>
       </c>
       <c r="P29" s="56">
         <f>IF(G29=0,0,N29/G29)</f>
-        <v>0.33181818181818185</v>
+        <v>0.1827272727272727</v>
       </c>
       <c r="Q29" s="56">
         <f>IF(G29=0,0,O29/G29)</f>
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="R29" s="54">
         <f>D29-M29</f>
@@ -6171,11 +6171,11 @@
       </c>
       <c r="S29" s="57">
         <f>IF(K29=0,0,O29/K29)</f>
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="T29" s="58">
         <f>G29-O29</f>
-        <v>176</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Align Cost report KPI fields to 01 DailyReport_TOTAL schema.
Manual Schedule/Progress entry now uses the Summary Phase Grand Total columns (Earned / Planned / Target Mhr, Earned % / Plan %, Inc Earned). PPR Earned prefers those KPIs and only falls back to expended=earned when they are blank (Day-0). Schema-only — the P66 DailyReport_TOTAL book stays on Drive, Slicer stays parked, SAMPLE refreshed with distinct earned vs expended.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
+++ b/look-samples/hit-squad-wood-river-sample-boiler-outage-ppr-2026-09-03.xlsx
@@ -52,7 +52,7 @@
             <sz val="9"/>
             <rFont val="Calibri"/>
           </rPr>
-          <t>Earned hours from scheduler KPI on Cost report. Physical % = earned / Direct budget hours (hours win if % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
+          <t>Earned Mhr from 01 DailyReport_TOTAL KPI on Cost report (Summary Phase Grand Total). Physical % = earned / Direct budget hours (hours win if Earned % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
         </r>
       </text>
     </comment>
@@ -300,7 +300,7 @@
     <t>TOTAL PROJECT</t>
   </si>
   <si>
-    <t>SAMPLE status — invented hours and dollars only  ·  Earned hours from scheduler KPI on Cost report. Physical % = earned / Direct budget hours (hours win if % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
+    <t>SAMPLE status — invented hours and dollars only  ·  Earned Mhr from 01 DailyReport_TOTAL KPI on Cost report (Summary Phase Grand Total). Physical % = earned / Direct budget hours (hours win if Earned % was also typed). Support earned = Direct % × Support budget hours. Budget from the live Hit Squad estimate pack — not Mike’s Estimate Summary links.</t>
   </si>
   <si>
     <t>Hours S-curve  ·  steel = live-pack estimate  ·  amber = T3 Export 16 spent</t>

</xml_diff>